<commit_message>
feat: add comprehensive WCAG-compliant Excel generation with openxlsx
- Implement create_openxlsx_accessible.R with full accessibility features
- Add multiple worksheet structure (GT_Table, Accessible_Data, Column_Mapping, Summary, Guide)
- Support both standard and high contrast color schemes for enhanced visibility
- Include proper table structure with screen reader optimization
- Add alternative text via cell comments for all headers
- Implement frozen panes and logical reading order
- Support complex German statistical data with special characters
- Add comprehensive test suite with 5 different test scenarios
- Include demo script showing professional usage examples
- Enhance formatted Excel generation with automatic vs manual formatting options
- Achieve WCAG 2.1 AA/AAA compliance with proper color contrast
- Support hierarchical spanner structures matching GT table appearance
</commit_message>
<xml_diff>
--- a/projects/r-accessible-tables/formatted_mikrozensus_sample.xlsx
+++ b/projects/r-accessible-tables/formatted_mikrozensus_sample.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="GT_Table" sheetId="1" r:id="rId1"/>
     <sheet name="Accessible_Data" sheetId="2" r:id="rId2"/>
-    <sheet name="Table_Info" sheetId="3" r:id="rId3"/>
+    <sheet name="Formatting_Instructions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -348,7 +348,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>German Mikrozensus - Clean GT Layout</t>
+          <t>German Mikrozensus - Professional Format</t>
         </is>
       </c>
     </row>
@@ -506,102 +506,102 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>OPENXLSX_RECOMMENDED</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>German Mikrozensus - Clean GT Layout</t>
+          <t>Install openxlsx package for automatic formatting</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Row 1, spans all columns</t>
+          <t>Run: install.packages('openxlsx') then use this script</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Structure_Type</t>
+          <t>1_TITLE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Multi-level with spanners</t>
+          <t>Select A1:E1 and merge cells</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Row 3: spanners, Row 4: headers</t>
+          <t>Title should span all columns with blue background (#366092)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Spanner Verheiratet</t>
+          <t>2_SPANNER_VERHEIRATET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Spans columns 1 to 2</t>
+          <t>Select A3:B3 and merge cells</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Row 3, columns 1-2</t>
+          <t>Spanner Verheiratet with blue background (#4F81BD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Spanner Single</t>
+          <t>2_SPANNER_SINGLE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Spans columns 3 to 4</t>
+          <t>Select C3:D3 and merge cells</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Row 3, columns 3-4</t>
+          <t>Spanner Single with blue background (#4F81BD)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Data_Location</t>
+          <t>3_HEADERS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2 data rows</t>
+          <t>Format row 4 as headers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Starting from row 6</t>
+          <t>Light blue background (#B7D4F0), bold text, borders</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Manual_Formatting</t>
+          <t>4_DATA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>To complete GT appearance, merge empty cells with spanner headers</t>
+          <t>Format data rows (6 onwards)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Use Excel merge cells function on appropriate ranges</t>
+          <t>Light borders, center alignment, auto-fit columns</t>
         </is>
       </c>
     </row>

</xml_diff>